<commit_message>
Split targets into one file per id, matching load_sut_from_parquet pattern
load_balancing_targets_from_excel now takes id_values and paths lists.
Each file has no id column — the loader inserts it from id_values.
Fixture ta_targets_2021.xlsx updated to drop the year column.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/fixtures/ta_targets_2021.xlsx
+++ b/data/fixtures/ta_targets_2021.xlsx
@@ -413,210 +413,172 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>year</t>
+          <t>trans</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>trans</t>
+          <t>brch</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>brch</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
           <t>maal</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>2021</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>0100</t>
+        </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
           <t>0100</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>0100</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>0700</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="n">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="D2" t="n">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>2021</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>0100</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
+      <c r="C6" t="n">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="D3" t="n">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>2021</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>0100</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Z</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>2021</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>0700</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="n">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>2021</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>2000</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>2021</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>2000</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
+      <c r="C7" t="n">
         <v>71</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
-        <v>2021</v>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>3110</t>
+        </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>3110</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
           <t>HH</t>
         </is>
       </c>
-      <c r="D8" t="n">
+      <c r="C8" t="n">
         <v>160</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
-        <v>2021</v>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>3200</t>
+        </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>3200</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
           <t>GOV</t>
         </is>
       </c>
-      <c r="D9" t="n">
+      <c r="C9" t="n">
         <v>65</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
-        <v>2021</v>
-      </c>
-      <c r="B10" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>5139</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="n">
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="n">
         <v>28</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
-        <v>2021</v>
-      </c>
-      <c r="B11" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>5200</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="n">
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="n">
         <v>32</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="n">
-        <v>2021</v>
-      </c>
-      <c r="B12" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>6001</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="n">
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="n">
         <v>58</v>
       </c>
     </row>

</xml_diff>